<commit_message>
Deterministic tie-break ordering in findings and Tableau queries; regenerate outputs
</commit_message>
<xml_diff>
--- a/tableau/hr_analytics_dashboard.xlsx
+++ b/tableau/hr_analytics_dashboard.xlsx
@@ -2740,16 +2740,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Neoplasms</t>
+          <t>Blood donation</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ICD disease</t>
+          <t>Non-ICD</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D21" t="n">
         <v>24</v>
@@ -2758,22 +2758,22 @@
         <v>0.5</v>
       </c>
       <c r="F21" t="n">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Blood donation</t>
+          <t>Neoplasms</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Non-ICD</t>
+          <t>ICD disease</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D22" t="n">
         <v>24</v>
@@ -2782,7 +2782,7 @@
         <v>0.5</v>
       </c>
       <c r="F22" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
     </row>
     <row r="23">
@@ -2860,7 +2860,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Congenital malformations</t>
+          <t>Blood and immune disorders</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -2884,7 +2884,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Blood and immune disorders</t>
+          <t>Congenital malformations</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">

</xml_diff>